<commit_message>
FIX on monitoring fetching
</commit_message>
<xml_diff>
--- a/test/fixtures/Consumption.xlsx
+++ b/test/fixtures/Consumption.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91983\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E280B488-CE63-4B16-BEE7-FD85DB696435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{80FF978B-A5B5-4115-921E-D25003F75A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" firstSheet="2" xr2:uid="{E31954A8-F205-4074-912D-A6C80DBF21DB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{E31954A8-F205-4074-912D-A6C80DBF21DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Consumption" sheetId="1" r:id="rId1"/>
@@ -76,7 +76,7 @@
     <t>Petrol</t>
   </si>
   <si>
-    <t>KwH</t>
+    <t>kWh</t>
   </si>
   <si>
     <t>Feb</t>
@@ -918,9 +918,6 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G15" xr:uid="{FD14E964-E8C7-4A4C-9D1F-3ED2593197F9}">
-      <formula1>"L,m3,kWh"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E15" xr:uid="{AD0CA9BE-9DFE-4884-BBA8-8ACD974BAF12}">
       <formula1>"Grid Electricity,Gas,Solar PV,Petrol,Diesel,Bio Diesel"</formula1>
     </dataValidation>
@@ -929,6 +926,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C15" xr:uid="{255F2D34-3163-4B59-AFEA-C99CC37DF630}">
       <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G15" xr:uid="{159F14B7-99E7-404E-8F18-C82C90DE0421}">
+      <formula1>"L,m3,kWh"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1011,7 +1011,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3" xr:uid="{B790D348-EC39-4664-B9A5-7B6386D03E52}">
       <formula1>"Grid Electricity,Gas,Solar PV,Petrol,Diesel,Bio Diesel"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{10923AFD-0165-41B8-9D52-215D757CAE0D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{BBDBD2E5-C267-414D-9DA8-57418F87B073}">
       <formula1>"L,m3,kWh"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1082,7 +1082,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{32FEFBA2-4084-4CA1-9746-B4B607554823}">
       <formula1>"Grid Electricity,Gas,Solar PV,Petrol,Diesel,Bio Diesel"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{E3F7DD02-63B7-46FD-AAB1-14A29E0EDC65}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{B4B939C5-8FBB-4B0E-8F8C-7F982799865C}">
       <formula1>"L,m3,kWh"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
FIX on utility import
</commit_message>
<xml_diff>
--- a/test/fixtures/Consumption.xlsx
+++ b/test/fixtures/Consumption.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91983\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80FF978B-A5B5-4115-921E-D25003F75A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CF01831-B462-4252-ABF2-0A03E3D7E94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{E31954A8-F205-4074-912D-A6C80DBF21DB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" firstSheet="2" activeTab="2" xr2:uid="{E31954A8-F205-4074-912D-A6C80DBF21DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Consumption" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="27">
   <si>
     <t>Site Code</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t>Conversion Factor</t>
+  </si>
+  <si>
+    <t>604_main_a</t>
   </si>
   <si>
     <t>Jan</t>
@@ -511,26 +514,26 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="15">
-      <c r="A2">
-        <v>604</v>
+      <c r="A2" t="s">
+        <v>9</v>
       </c>
       <c r="B2">
         <v>2023</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2">
         <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H2">
         <v>200</v>
@@ -540,26 +543,26 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="15">
-      <c r="A3">
-        <v>604</v>
+      <c r="A3" t="s">
+        <v>9</v>
       </c>
       <c r="B3">
         <v>2023</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3">
         <v>120</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H3">
         <v>300</v>
@@ -569,26 +572,26 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="15">
-      <c r="A4">
-        <v>604</v>
+      <c r="A4" t="s">
+        <v>9</v>
       </c>
       <c r="B4">
         <v>2023</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4">
         <v>200</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H4">
         <v>400</v>
@@ -598,26 +601,26 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="15">
-      <c r="A5">
-        <v>604</v>
+      <c r="A5" t="s">
+        <v>9</v>
       </c>
       <c r="B5">
         <v>2023</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5">
         <v>120</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H5">
         <v>300</v>
@@ -627,26 +630,26 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="15">
-      <c r="A6">
-        <v>604</v>
+      <c r="A6" t="s">
+        <v>9</v>
       </c>
       <c r="B6">
         <v>2023</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6">
         <v>200</v>
       </c>
       <c r="G6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H6">
         <v>400</v>
@@ -656,26 +659,26 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="15">
-      <c r="A7">
-        <v>604</v>
+      <c r="A7" t="s">
+        <v>9</v>
       </c>
       <c r="B7">
         <v>2023</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7">
         <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H7">
         <v>300</v>
@@ -685,26 +688,26 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="15">
-      <c r="A8">
-        <v>604</v>
+      <c r="A8" t="s">
+        <v>9</v>
       </c>
       <c r="B8">
         <v>2023</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8">
         <v>200</v>
       </c>
       <c r="G8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H8">
         <v>400</v>
@@ -714,26 +717,26 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="15">
-      <c r="A9">
-        <v>604</v>
+      <c r="A9" t="s">
+        <v>9</v>
       </c>
       <c r="B9">
         <v>2023</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F9">
         <v>120</v>
       </c>
       <c r="G9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H9">
         <v>300</v>
@@ -743,26 +746,26 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="15">
-      <c r="A10">
-        <v>604</v>
+      <c r="A10" t="s">
+        <v>9</v>
       </c>
       <c r="B10">
         <v>2023</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F10">
         <v>200</v>
       </c>
       <c r="G10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H10">
         <v>400</v>
@@ -772,26 +775,26 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="15">
-      <c r="A11">
-        <v>604</v>
+      <c r="A11" t="s">
+        <v>9</v>
       </c>
       <c r="B11">
         <v>2023</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F11">
         <v>120</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H11">
         <v>300</v>
@@ -801,26 +804,26 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="15">
-      <c r="A12">
-        <v>604</v>
+      <c r="A12" t="s">
+        <v>9</v>
       </c>
       <c r="B12">
         <v>2023</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F12">
         <v>200</v>
       </c>
       <c r="G12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H12">
         <v>400</v>
@@ -830,26 +833,26 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="15">
-      <c r="A13">
-        <v>604</v>
+      <c r="A13" t="s">
+        <v>9</v>
       </c>
       <c r="B13">
         <v>2023</v>
       </c>
       <c r="C13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13">
         <v>120</v>
       </c>
       <c r="G13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H13">
         <v>300</v>
@@ -859,26 +862,26 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="15">
-      <c r="A14">
-        <v>604</v>
+      <c r="A14" t="s">
+        <v>9</v>
       </c>
       <c r="B14">
         <v>2022</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F14">
         <v>200</v>
       </c>
       <c r="G14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H14">
         <v>400</v>
@@ -888,26 +891,26 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="15">
-      <c r="A15">
-        <v>604</v>
+      <c r="A15" t="s">
+        <v>9</v>
       </c>
       <c r="B15">
         <v>2022</v>
       </c>
       <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="E15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F15">
         <v>120</v>
       </c>
       <c r="G15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H15">
         <v>300</v>
@@ -960,44 +963,44 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2">
-        <v>604</v>
+      <c r="A2" t="s">
+        <v>9</v>
       </c>
       <c r="B2">
         <v>2023</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2">
         <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3">
-        <v>604</v>
+      <c r="A3" t="s">
+        <v>9</v>
       </c>
       <c r="B3">
         <v>2023</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3">
         <v>1.5</v>
@@ -1045,27 +1048,27 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2">
-        <v>604</v>
+      <c r="A2" t="s">
+        <v>9</v>
       </c>
       <c r="B2">
         <v>2023</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2">
         <v>20</v>

</xml_diff>

<commit_message>
REFACTOR on patters import
</commit_message>
<xml_diff>
--- a/test/fixtures/Consumption.xlsx
+++ b/test/fixtures/Consumption.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91983\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CF01831-B462-4252-ABF2-0A03E3D7E94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AAD8A54-D7F1-4ACA-9538-9C3BCBE54033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" firstSheet="2" activeTab="2" xr2:uid="{E31954A8-F205-4074-912D-A6C80DBF21DB}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="28">
   <si>
     <t>Site Code</t>
   </si>
@@ -100,19 +100,22 @@
     <t>May</t>
   </si>
   <si>
+    <t>m3</t>
+  </si>
+  <si>
     <t>Jun</t>
   </si>
   <si>
     <t>Cooling</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>Dec</t>
   </si>
   <si>
     <t>Emission Factor</t>
-  </si>
-  <si>
-    <t>L</t>
   </si>
   <si>
     <t xml:space="preserve">Target Energy </t>
@@ -649,7 +652,7 @@
         <v>200</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H6">
         <v>400</v>
@@ -666,7 +669,7 @@
         <v>2023</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>11</v>
@@ -698,7 +701,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -727,7 +730,7 @@
         <v>14</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
@@ -756,7 +759,7 @@
         <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
         <v>12</v>
@@ -765,7 +768,7 @@
         <v>200</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="H10">
         <v>400</v>
@@ -785,7 +788,7 @@
         <v>18</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s">
         <v>12</v>
@@ -814,7 +817,7 @@
         <v>19</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
         <v>12</v>
@@ -840,10 +843,10 @@
         <v>2023</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>
@@ -869,7 +872,7 @@
         <v>2022</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>11</v>
@@ -898,10 +901,10 @@
         <v>2022</v>
       </c>
       <c r="C15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="E15" t="s">
         <v>15</v>
@@ -963,7 +966,7 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1000,7 +1003,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F3">
         <v>1.5</v>
@@ -1048,10 +1051,10 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:7">

</xml_diff>

<commit_message>
REFACTOR on site import and consumption, emission, monitoring import
</commit_message>
<xml_diff>
--- a/test/fixtures/Consumption.xlsx
+++ b/test/fixtures/Consumption.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91983\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AAD8A54-D7F1-4ACA-9538-9C3BCBE54033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09540FF3-5757-4E53-B2E3-85EB23B19664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" firstSheet="2" activeTab="2" xr2:uid="{E31954A8-F205-4074-912D-A6C80DBF21DB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{E31954A8-F205-4074-912D-A6C80DBF21DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Consumption" sheetId="1" r:id="rId1"/>
@@ -542,7 +542,7 @@
         <v>200</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15">
@@ -571,7 +571,7 @@
         <v>300</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15">
@@ -600,7 +600,7 @@
         <v>400</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15">
@@ -629,7 +629,7 @@
         <v>300</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15">
@@ -658,7 +658,7 @@
         <v>400</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15">
@@ -687,7 +687,7 @@
         <v>300</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15">
@@ -716,7 +716,7 @@
         <v>400</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15">
@@ -733,10 +733,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F9">
-        <v>120</v>
+        <v>84.69</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -745,7 +745,7 @@
         <v>300</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15">
@@ -765,7 +765,7 @@
         <v>12</v>
       </c>
       <c r="F10">
-        <v>200</v>
+        <v>263.33999999999997</v>
       </c>
       <c r="G10" t="s">
         <v>23</v>
@@ -774,7 +774,7 @@
         <v>400</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15">
@@ -803,7 +803,7 @@
         <v>300</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15">
@@ -832,7 +832,7 @@
         <v>400</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15">
@@ -861,7 +861,7 @@
         <v>300</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15">
@@ -890,7 +890,7 @@
         <v>400</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15">
@@ -919,7 +919,7 @@
         <v>300</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>25.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>